<commit_message>
Updated Text To Dolumn.xlsx
</commit_message>
<xml_diff>
--- a/Text To Dolumn.xlsx
+++ b/Text To Dolumn.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Besant\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63C85E82-2F1D-460E-B459-3CF12E0571D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A41D324-1BEF-47B0-A9DE-C5DFC1FDF520}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{36344CCA-E400-46A8-8EFA-5E6271D0DEB8}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="85">
   <si>
     <t>DATA</t>
   </si>
@@ -190,6 +190,105 @@
   </si>
   <si>
     <t>then click finish</t>
+  </si>
+  <si>
+    <t>Employee Name</t>
+  </si>
+  <si>
+    <t>JP Kumar</t>
+  </si>
+  <si>
+    <t>Anjali ,Thakur</t>
+  </si>
+  <si>
+    <t>"Priya AgarwaL"</t>
+  </si>
+  <si>
+    <t>R#Vasu,Muthanna</t>
+  </si>
+  <si>
+    <t>Sanjay;Gupta</t>
+  </si>
+  <si>
+    <t>Jharna ,Biswal</t>
+  </si>
+  <si>
+    <t>Prakash#Dutta</t>
+  </si>
+  <si>
+    <t>Manisha;Guha</t>
+  </si>
+  <si>
+    <t>Arjun,JAiN</t>
+  </si>
+  <si>
+    <t>Arjun#Kapoor</t>
+  </si>
+  <si>
+    <t>"Ajay Kumar"</t>
+  </si>
+  <si>
+    <t>JP</t>
+  </si>
+  <si>
+    <t>Kumar</t>
+  </si>
+  <si>
+    <t>Anjali</t>
+  </si>
+  <si>
+    <t>Thakur</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>Vasu</t>
+  </si>
+  <si>
+    <t>Muthanna</t>
+  </si>
+  <si>
+    <t>Sanjay</t>
+  </si>
+  <si>
+    <t>Gupta</t>
+  </si>
+  <si>
+    <t>Jharna</t>
+  </si>
+  <si>
+    <t>Biswal</t>
+  </si>
+  <si>
+    <t>Prakash</t>
+  </si>
+  <si>
+    <t>Dutta</t>
+  </si>
+  <si>
+    <t>Manisha</t>
+  </si>
+  <si>
+    <t>Guha</t>
+  </si>
+  <si>
+    <t>Arjun</t>
+  </si>
+  <si>
+    <t>JAiN</t>
+  </si>
+  <si>
+    <t>Kapoor</t>
+  </si>
+  <si>
+    <t>Priya</t>
+  </si>
+  <si>
+    <t>AgarwaL</t>
+  </si>
+  <si>
+    <t>Ajay</t>
   </si>
 </sst>
 </file>
@@ -233,9 +332,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -550,20 +652,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1359D29E-5012-443A-8E74-4ED2366FB76C}">
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:Q24"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="37.6328125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="25.26953125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="37.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="N1" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -594,8 +700,17 @@
       <c r="L2">
         <v>8562</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="N2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="O2" t="s">
+        <v>64</v>
+      </c>
+      <c r="P2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -626,8 +741,17 @@
       <c r="L3">
         <v>9845</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="N3" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="O3" t="s">
+        <v>66</v>
+      </c>
+      <c r="P3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -658,8 +782,17 @@
       <c r="L4">
         <v>9878</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="N4" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="O4" t="s">
+        <v>82</v>
+      </c>
+      <c r="P4" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -690,8 +823,20 @@
       <c r="L5">
         <v>2378</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="N5" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="O5" t="s">
+        <v>68</v>
+      </c>
+      <c r="P5" t="s">
+        <v>69</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -722,8 +867,17 @@
       <c r="L6">
         <v>9567</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="N6" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="O6" t="s">
+        <v>71</v>
+      </c>
+      <c r="P6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -754,8 +908,17 @@
       <c r="L7">
         <v>8923</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="N7" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="O7" t="s">
+        <v>73</v>
+      </c>
+      <c r="P7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -786,8 +949,17 @@
       <c r="L8">
         <v>5679</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="N8" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="O8" t="s">
+        <v>75</v>
+      </c>
+      <c r="P8" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -818,8 +990,17 @@
       <c r="L9">
         <v>7453</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="N9" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="O9" t="s">
+        <v>77</v>
+      </c>
+      <c r="P9" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -850,8 +1031,17 @@
       <c r="L10">
         <v>4598</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="N10" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="O10" t="s">
+        <v>79</v>
+      </c>
+      <c r="P10" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -882,8 +1072,17 @@
       <c r="L11">
         <v>8345</v>
       </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="N11" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="O11" t="s">
+        <v>79</v>
+      </c>
+      <c r="P11" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -914,54 +1113,93 @@
       <c r="L12">
         <v>3456</v>
       </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="N12" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="O12" t="s">
+        <v>84</v>
+      </c>
+      <c r="P12" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="N15" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="N16" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="N17" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="N18" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="N19" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="N20" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="N21" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="N22" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="N23" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
+        <v>51</v>
+      </c>
+      <c r="N24" s="2" t="s">
         <v>51</v>
       </c>
     </row>

</xml_diff>